<commit_message>
Update videos, width baseline & fonts
</commit_message>
<xml_diff>
--- a/六元_作品时间轴.xlsx
+++ b/六元_作品时间轴.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python练习\六元\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED2C0EA-A279-42CD-AF40-21A5A2FDBE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD66ED5-E0F1-48DA-BBC5-C0A96D55F9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{7D1B2066-D2B7-4F32-9662-CD01F844A157}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="183">
   <si>
     <t>作品</t>
   </si>
@@ -668,6 +668,30 @@
   </si>
   <si>
     <t>我想完成一次...完美的犯罪</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\海岛舒服日志_1.mp4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\海岛舒服日志_2.mp4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\海岛舒服日志_3.mp4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\我的朋友安德烈_1.mp4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\我的朋友安德烈_2.mp4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\python练习\六元\我的朋友安德烈_3.mp4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1901,13 +1925,13 @@
         <v>81</v>
       </c>
       <c r="I22" t="s">
-        <v>98</v>
+        <v>180</v>
       </c>
       <c r="J22" t="s">
-        <v>97</v>
+        <v>181</v>
       </c>
       <c r="K22" t="s">
-        <v>99</v>
+        <v>182</v>
       </c>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -1974,13 +1998,13 @@
         <v>82</v>
       </c>
       <c r="I24" t="s">
-        <v>98</v>
+        <v>177</v>
       </c>
       <c r="J24" t="s">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="K24" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.4">

</xml_diff>